<commit_message>
📊 Horarios actualizados Línea 141 - 5140
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:25</t>
+          <t>Última actualización: 06:26:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>105</v>
+        <v>8</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,398 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:52</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>109</v>
+        <v>13</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>13</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:56</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>33</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>53</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>54</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>55</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>61</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>69</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>69</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>71</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>89</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>105</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>111</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:25</t>
+          <t>Última actualización: 06:26:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -610,21 +985,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -635,23 +1010,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:52</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -668,7 +1068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -681,14 +1081,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:25</t>
+          <t>Última actualización: 06:26:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:26:03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>78</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5141
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:03</t>
+          <t>Última actualización: 10:25:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -915,6 +915,581 @@
         <v>111</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>18</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>19</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>26</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>30</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>31</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>33</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>37</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>45</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>48</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>49</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>11:16</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>51</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>55</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>60</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>62</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>73</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>77</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>78</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>88</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>93</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>103</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>108</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -931,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,14 +1519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:03</t>
+          <t>Última actualización: 10:25:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1052,6 +1627,56 @@
         <v>69</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>73</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1068,7 +1693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,14 +1706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:03</t>
+          <t>Última actualización: 10:25:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1141,6 +1766,81 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10:25:49</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5142
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:25:49</t>
+          <t>Última actualización: 13:45:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 61</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1490,6 +1490,506 @@
         <v>108</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>23</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>23</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>27</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>32</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>40</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>42</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>43</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>56</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>63</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>70</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>72</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>81</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>82</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>15:08</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>83</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>85</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>86</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>102</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>103</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1506,7 +2006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1519,14 +2019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:25:49</t>
+          <t>Última actualización: 13:45:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1677,6 +2177,106 @@
         <v>73</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>43</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>63</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>72</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>103</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1693,7 +2293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1706,14 +2306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:25:49</t>
+          <t>Última actualización: 13:45:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1841,6 +2441,81 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>43</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>13:45:02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>88</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5143
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:02</t>
+          <t>Última actualización: 16:02:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 61</t>
+          <t>Total filas: 80</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1990,6 +1990,481 @@
         <v>103</v>
       </c>
       <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>5</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>9</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>21</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>23</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>25</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>36</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>38</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>38</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>39</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>39</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>51</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>66</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>80</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>88</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>91</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>94</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>96</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>108</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>116</v>
+      </c>
+      <c r="E85" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2006,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2019,14 +2494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:02</t>
+          <t>Última actualización: 16:02:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2277,6 +2752,81 @@
         <v>103</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>66</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>91</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>17:58</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>116</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2293,7 +2843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2306,14 +2856,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:45:02</t>
+          <t>Última actualización: 16:02:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2516,6 +3066,81 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>36</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>16:02:11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>61</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5144
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:02:11</t>
+          <t>Última actualización: 18:31:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 80</t>
+          <t>Total filas: 101</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2465,6 +2465,531 @@
         <v>116</v>
       </c>
       <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>5</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>6</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>22</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>34</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>37</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>40</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>46</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>50</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>52</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>55</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>69</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>70</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>72</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>92</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>92</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>99</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>112</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>114</v>
+      </c>
+      <c r="E106" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2481,7 +3006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2494,14 +3019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:02:11</t>
+          <t>Última actualización: 18:31:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2827,6 +3352,81 @@
         <v>116</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>37</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>52</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>92</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2843,7 +3443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2856,14 +3456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:02:11</t>
+          <t>Última actualización: 18:31:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -3139,6 +3739,81 @@
         <v>61</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>31</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>18:31:17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>91</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5145
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:31:17</t>
+          <t>Última actualización: 20:37:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 101</t>
+          <t>Total filas: 115</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2990,6 +2990,356 @@
         <v>114</v>
       </c>
       <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>4</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>8</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>14</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>19</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>25</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>33</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>49</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>57</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>59</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>63</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>69</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>87</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>98</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>116</v>
+      </c>
+      <c r="E120" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3006,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3019,14 +3369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:31:17</t>
+          <t>Última actualización: 20:37:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3427,6 +3777,56 @@
         <v>92</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>116</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3443,7 +3843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3456,14 +3856,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:31:17</t>
+          <t>Última actualización: 20:37:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3816,6 +4216,81 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>49</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20:37:31</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>99</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5146
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-24.xlsx
+++ b/data/horarios-141-2026-10-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E120"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:37:31</t>
+          <t>Última actualización: 22:33:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 115</t>
+          <t>Total filas: 123</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:26:03</t>
+          <t>22:33:52</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>00:12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>99</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -503,16 +503,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -528,16 +528,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -578,16 +578,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:56</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -628,16 +628,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -653,16 +653,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -678,16 +678,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -703,16 +703,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,16 +753,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -828,16 +828,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -878,16 +878,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -903,16 +903,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10:25:49</t>
+          <t>06:26:03</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>111</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -978,16 +978,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:27</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1028,16 +1028,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1128,16 +1128,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1178,16 +1178,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,16 +1228,16 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11:16</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,16 +1253,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:16</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1303,16 +1303,16 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1328,16 +1328,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>11:43</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:43</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1428,16 +1428,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,16 +1478,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>13:45:02</t>
+          <t>10:25:49</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1553,16 +1553,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1653,16 +1653,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1678,16 +1678,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1803,16 +1803,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1828,16 +1828,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>15:08</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1903,16 +1903,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:08</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,16 +1928,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>16:02:11</t>
+          <t>13:45:02</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5</v>
+        <v>103</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2028,16 +2028,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2078,16 +2078,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2153,16 +2153,16 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2203,16 +2203,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2253,16 +2253,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2303,16 +2303,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2328,16 +2328,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2353,16 +2353,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2378,16 +2378,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>17:58</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>18:31:17</t>
+          <t>16:02:11</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>17:58</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>18:32</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:32</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2578,16 +2578,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2628,16 +2628,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,16 +2703,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2728,16 +2728,16 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2853,16 +2853,16 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2878,16 +2878,16 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2953,16 +2953,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2978,16 +2978,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>20:37:31</t>
+          <t>18:31:17</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>4</v>
+        <v>114</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3028,16 +3028,16 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3078,16 +3078,16 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3178,16 +3178,16 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3253,16 +3253,16 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>22:04</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>22:15</t>
+          <t>22:04</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3328,18 +3328,218 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>98</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
           <t>22:33</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D120" t="n">
-        <v>116</v>
-      </c>
-      <c r="E120" t="inlineStr">
+      <c r="D122" t="n">
+        <v>0</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>2</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>12</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>23:03</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>30</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>23:18</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>45</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>66</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>23:58</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>85</v>
+      </c>
+      <c r="E128" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3356,7 +3556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3369,14 +3569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:37:31</t>
+          <t>Última actualización: 22:33:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3810,7 +4010,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>20:37:31</t>
+          <t>22:33:52</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3824,9 +4024,34 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22:33:52</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>66</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3856,7 +4081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:37:31</t>
+          <t>Última actualización: 22:33:52</t>
         </is>
       </c>
     </row>

</xml_diff>